<commit_message>
HRIS project v 0.0.33
</commit_message>
<xml_diff>
--- a/public/template/template_upload_karyawan.xlsx
+++ b/public/template/template_upload_karyawan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ict-d\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\project\hris-prod\public\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E10A50CC-078F-448B-B9F6-A2B578EEBEEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9874FAD9-2ABA-48F9-8A80-91A77A0A7432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{9D850D6C-A414-4510-85CE-67383360A39D}"/>
+    <workbookView xWindow="-108" yWindow="444" windowWidth="23256" windowHeight="12624" xr2:uid="{9D850D6C-A414-4510-85CE-67383360A39D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="83">
   <si>
     <t>Ex : Karawang</t>
   </si>
@@ -238,6 +238,51 @@
   </si>
   <si>
     <t>Tanggal Bergabung (dd/mm/yyyy)</t>
+  </si>
+  <si>
+    <t>Tipe  Karyawan (String)</t>
+  </si>
+  <si>
+    <t>Status Kawin (String)</t>
+  </si>
+  <si>
+    <t>Hubungan Pasangan (String)</t>
+  </si>
+  <si>
+    <t>Nama Pasangan (String)</t>
+  </si>
+  <si>
+    <t>Tempat Lahir Pasangan (String)</t>
+  </si>
+  <si>
+    <t>Tangal Lahir Pasangan (dd/mm/yyyy)</t>
+  </si>
+  <si>
+    <t>Hubungan Anak ()</t>
+  </si>
+  <si>
+    <t>Anak 1</t>
+  </si>
+  <si>
+    <t>Nama Anak (String)</t>
+  </si>
+  <si>
+    <t>Tempat Lahir Anak (String)</t>
+  </si>
+  <si>
+    <t>Tangal Lahir Anak (dd/mm/yyyy)</t>
+  </si>
+  <si>
+    <t>Anak 2</t>
+  </si>
+  <si>
+    <t>Anak 3</t>
+  </si>
+  <si>
+    <t>Anak 4</t>
+  </si>
+  <si>
+    <t>Anak 5</t>
   </si>
 </sst>
 </file>
@@ -648,48 +693,74 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69D0E4EC-B375-444C-A099-75B908B6C530}">
-  <dimension ref="A1:AK4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:BK2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="47.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="94.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="52.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="45.1796875" customWidth="1"/>
-    <col min="5" max="5" width="29.81640625" customWidth="1"/>
+    <col min="1" max="1" width="47.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="94.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="52.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="45.21875" customWidth="1"/>
+    <col min="5" max="5" width="29.77734375" customWidth="1"/>
     <col min="6" max="7" width="33" customWidth="1"/>
-    <col min="8" max="8" width="29.08984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="49.81640625" customWidth="1"/>
-    <col min="10" max="10" width="38.26953125" customWidth="1"/>
+    <col min="8" max="8" width="29.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="49.77734375" customWidth="1"/>
+    <col min="10" max="10" width="38.21875" customWidth="1"/>
     <col min="11" max="11" width="32" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="80" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="31.81640625" customWidth="1"/>
-    <col min="14" max="14" width="76.81640625" customWidth="1"/>
-    <col min="15" max="15" width="34.26953125" customWidth="1"/>
-    <col min="16" max="16" width="43.08984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="35.81640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="31.453125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="37.90625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="36.81640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="37.1796875" customWidth="1"/>
+    <col min="13" max="13" width="31.77734375" customWidth="1"/>
+    <col min="14" max="14" width="76.77734375" customWidth="1"/>
+    <col min="15" max="15" width="34.21875" customWidth="1"/>
+    <col min="16" max="16" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="35.77734375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="31.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="37.88671875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="36.77734375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="37.21875" customWidth="1"/>
     <col min="22" max="22" width="36" customWidth="1"/>
-    <col min="23" max="23" width="33.26953125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="37.6328125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="27.54296875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="35.6328125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="28.54296875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="52.54296875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="37.81640625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="40.36328125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="31.08984375" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="32.81640625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="34.90625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="37.453125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="48.90625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="29.7265625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="31.1796875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="33.21875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="37.6640625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="27.5546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="28.5546875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="52.5546875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="37.77734375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="40.33203125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="31.109375" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="32.77734375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="34.88671875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="37.44140625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="48.88671875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="29.77734375" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="31.21875" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="29" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="24.77734375" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="32.6640625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="27.88671875" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="36.33203125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="48.88671875" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="32.6640625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="27.88671875" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="36.33203125" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="41.6640625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="31.109375" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="36.44140625" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="31.109375" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="36.44140625" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="31.109375" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="36.44140625" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="31.109375" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="36.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="17" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:63" ht="17.399999999999999" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>43</v>
       </c>
@@ -801,8 +872,86 @@
       <c r="AK1" s="2" t="s">
         <v>65</v>
       </c>
+      <c r="AL1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM1" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AN1" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="AO1" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="AP1" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="AQ1" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="AR1" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AS1" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="AT1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AU1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AV1" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AW1" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="AX1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AY1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AZ1" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="BA1" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="BB1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="BC1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="BD1" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="BE1" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="BF1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="BG1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="BH1" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="BI1" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="BJ1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="BK1" s="4" t="s">
+        <v>78</v>
+      </c>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -914,13 +1063,20 @@
       <c r="AK2" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
-      <c r="Y4">
-        <v>24</v>
-      </c>
-      <c r="AF4">
-        <v>31</v>
+      <c r="AR2" t="s">
+        <v>75</v>
+      </c>
+      <c r="AV2" t="s">
+        <v>79</v>
+      </c>
+      <c r="AZ2" t="s">
+        <v>80</v>
+      </c>
+      <c r="BD2" t="s">
+        <v>81</v>
+      </c>
+      <c r="BH2" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
HRIS project v 0.0.35
</commit_message>
<xml_diff>
--- a/public/template/template_upload_karyawan.xlsx
+++ b/public/template/template_upload_karyawan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\project\hris-prod\public\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9874FAD9-2ABA-48F9-8A80-91A77A0A7432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BABC43F6-F3C0-4E1E-995E-6DBBD65DE6C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="444" windowWidth="23256" windowHeight="12624" xr2:uid="{9D850D6C-A414-4510-85CE-67383360A39D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="82">
   <si>
     <t>Ex : Karawang</t>
   </si>
@@ -54,9 +54,6 @@
     <t>Ex : O / A / B / AB</t>
   </si>
   <si>
-    <t>Ex : FATHAN PEBRI (Gunakan Huruf Kapital)</t>
-  </si>
-  <si>
     <t>Ex : 09.254.294.3-407.000</t>
   </si>
   <si>
@@ -66,24 +63,12 @@
     <t>Ex : 628987336533</t>
   </si>
   <si>
-    <t>Ex : 480.030524</t>
-  </si>
-  <si>
-    <t>Ex : FA1722</t>
-  </si>
-  <si>
-    <t>Ex : passwordakun123</t>
-  </si>
-  <si>
     <t>Ex : 17/02/2002</t>
   </si>
   <si>
     <t>Ex : 01/01/2024</t>
   </si>
   <si>
-    <t>Ex : Jl.Tricentrum No.2025</t>
-  </si>
-  <si>
     <t>Ex : MENIKAH / BELUM MENIKAH / CERAI</t>
   </si>
   <si>
@@ -283,6 +268,18 @@
   </si>
   <si>
     <t>Anak 5</t>
+  </si>
+  <si>
+    <t>Ex : 3822-0001</t>
+  </si>
+  <si>
+    <t>Ex : Jl.Surotokunto No.2025</t>
+  </si>
+  <si>
+    <t>Ex : ADHI NUR FAJAR (Gunakan Huruf Kapital)</t>
+  </si>
+  <si>
+    <t>Ex : 3821-0001</t>
   </si>
 </sst>
 </file>
@@ -762,270 +759,270 @@
   <sheetData>
     <row r="1" spans="1:63" ht="17.399999999999999" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="V1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="W1" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="I1" s="2" t="s">
+      <c r="Y1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="Z1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="AA1" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB1" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="AC1" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="AD1" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="AE1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF1" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AG1" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="AH1" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI1" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="AJ1" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="AM1" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="AN1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AO1" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="J1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="R1" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="S1" s="4" t="s">
+      <c r="AP1" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="T1" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="Y1" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="Z1" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="AA1" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB1" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="AC1" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="AD1" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="AE1" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AF1" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="AG1" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="AH1" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="AI1" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="AJ1" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="AK1" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AQ1" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AR1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AN1" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="AO1" s="2" t="s">
+      <c r="AS1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AT1" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AQ1" s="4" t="s">
+      <c r="AU1" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="AR1" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="AS1" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="AT1" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="AU1" s="4" t="s">
-        <v>78</v>
-      </c>
       <c r="AV1" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="AW1" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="AX1" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AY1" s="4" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AZ1" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="BA1" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="BB1" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="BC1" s="4" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="BD1" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="BE1" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="BF1" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="BG1" s="4" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="BH1" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="BI1" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="BJ1" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="BK1" s="4" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="E2" t="s">
         <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>79</v>
       </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>79</v>
       </c>
       <c r="H2" t="s">
         <v>0</v>
       </c>
       <c r="I2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="J2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="K2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="L2" t="s">
         <v>3</v>
       </c>
       <c r="M2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="N2" t="s">
         <v>2</v>
       </c>
       <c r="O2" t="s">
+        <v>6</v>
+      </c>
+      <c r="P2" t="s">
         <v>7</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
+        <v>7</v>
+      </c>
+      <c r="R2" t="s">
         <v>8</v>
       </c>
-      <c r="Q2" t="s">
-        <v>8</v>
-      </c>
-      <c r="R2" t="s">
-        <v>9</v>
-      </c>
       <c r="S2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="T2" t="s">
+        <v>13</v>
+      </c>
+      <c r="U2" t="s">
         <v>14</v>
       </c>
-      <c r="T2" t="s">
-        <v>18</v>
-      </c>
-      <c r="U2" t="s">
-        <v>19</v>
-      </c>
       <c r="V2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="W2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="X2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="Y2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="Z2" t="s">
         <v>1</v>
@@ -1034,49 +1031,49 @@
         <v>5</v>
       </c>
       <c r="AB2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="AC2" t="s">
-        <v>11</v>
+        <v>81</v>
       </c>
       <c r="AD2" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
       <c r="AE2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="AF2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="AG2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="AH2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="AI2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="AJ2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="AK2" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="AR2" t="s">
+        <v>70</v>
+      </c>
+      <c r="AV2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AZ2" t="s">
         <v>75</v>
       </c>
-      <c r="AV2" t="s">
-        <v>79</v>
-      </c>
-      <c r="AZ2" t="s">
-        <v>80</v>
-      </c>
       <c r="BD2" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="BH2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>